<commit_message>
Three more automations done just one left
</commit_message>
<xml_diff>
--- a/1-Manual Test Plans/PARADOX Website Test Plan – Version 1.0.xlsx
+++ b/1-Manual Test Plans/PARADOX Website Test Plan – Version 1.0.xlsx
@@ -8,15 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\dario\Documents\GitHub\ParadoxQATest_DarioSC\1-Manual Test Plans\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CD58931C-0BEC-4436-B69F-5A3E0A6E0FE3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{498684E7-CF3C-4236-A0A3-8A9981E1ABDA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="TestCases" sheetId="1" r:id="rId1"/>
+    <sheet name="TestPlan-NoLogIn" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">TestCases!$A$1:$I$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'TestPlan-NoLogIn'!$A$1:$I$1</definedName>
   </definedNames>
   <calcPr calcId="0"/>
   <extLst>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="133" uniqueCount="95">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="128" uniqueCount="91">
   <si>
     <t>TC ID</t>
   </si>
@@ -183,15 +183,6 @@
     <t>Search bar test</t>
   </si>
   <si>
-    <t>1.- Open [https://www.paradoxinteractive.com/our-games/all-games]
-2.- Click into the [SEARCH] bar and write the name of a PARADOX game
-3.- Click into the [SEARCH] bar and write the name of a non-Paradox game</t>
-  </si>
-  <si>
-    <t>2.- All games related to that title will be displayed
-3.- The "No matching games" message will appear, with no games displayed</t>
-  </si>
-  <si>
     <t>AllGames_02</t>
   </si>
   <si>
@@ -275,9 +266,6 @@
     <t>OnSale_01</t>
   </si>
   <si>
-    <t>On sale tag display test</t>
-  </si>
-  <si>
     <t>1.- Open [https://www.paradoxinteractive.com/our-games/on-sale]
 2.- Review all the games on the On Sale site</t>
   </si>
@@ -285,23 +273,7 @@
     <t>YourCart_01</t>
   </si>
   <si>
-    <t>Multiple add to cart test</t>
-  </si>
-  <si>
-    <t>1.- Open [https://www.paradoxinteractive.com/our-games/all-games]
-2.- Add to cart more than one game</t>
-  </si>
-  <si>
-    <t>2.- The games will be added to the cart normally. A pop-up will confirm each game as it is added</t>
-  </si>
-  <si>
-    <t>RP-1310263</t>
-  </si>
-  <si>
     <t>YourCart_02</t>
-  </si>
-  <si>
-    <t>Cart logical operations test</t>
   </si>
   <si>
     <t>1.- Open [https://www.paradoxinteractive.com/our-games/all-games]
@@ -310,11 +282,6 @@
 4.- Add one on sale game to the cart
 5.- Open the cart by clicking in the [🛒] button
 6.- Delete the on sale game</t>
-  </si>
-  <si>
-    <t>2. &amp; 4.- The games will be added to the cart normally. A pop-up will confirm each game as it is added
-5.- The cart page will open, displaying the selected games and the purchase summary with the sale price applied
-6.- The cart will update automatically to show the number of games and the purchase summary</t>
   </si>
   <si>
     <t>YourCart_03</t>
@@ -368,9 +335,6 @@
 (This is an example of what happens when a test case is designed but the feature cannot be tested. This test case should be marked Pass.)</t>
   </si>
   <si>
-    <t>YourCart_05</t>
-  </si>
-  <si>
     <t>Checkout options test</t>
   </si>
   <si>
@@ -396,6 +360,33 @@
   </si>
   <si>
     <t>&gt; There must not be any game in the cart</t>
+  </si>
+  <si>
+    <t>2. &amp; 4.- A pop-up should confirm that the games has been added to the cart, and the [🛒] button will show the number of games added
+5.- The cart page will open, displaying the selected games and the purchase summary with the sale price applied
+6.- The cart will update automatically to show the number of games and the purchase summary</t>
+  </si>
+  <si>
+    <t>Esential cart functions test</t>
+  </si>
+  <si>
+    <t>AUTOMIZED TEST: This test was automti</t>
+  </si>
+  <si>
+    <t>On sale tag display test</t>
+  </si>
+  <si>
+    <t>2.- The "No matching games" message will appear, with no games displayed
+3.- The text just inserted in the [SEARCH] bar will be deleted
+4.- All games related to that title will be displayed
+5.- A pop-up should confirm that the game has been added to the cart, and the [🛒] button will show the number of games added</t>
+  </si>
+  <si>
+    <t>1.- Open [https://www.paradoxinteractive.com/our-games/all-games]
+2.- Click into the [SEARCH] bar and write the name of a non-Paradox game (repeat this step for five times with non-PARADOX games)
+3.- Click into the [X] and [CLEAR ALL (X)] buton in the [SEARCH] bar 
+4.- Click into the [SEARCH] bar and write the name of a PARADOX game (repeat this step for five times with PARADOX games)
+5.- Add all the searched games to the cart</t>
   </si>
 </sst>
 </file>
@@ -518,10 +509,10 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -819,7 +810,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:I23"/>
+  <dimension ref="A1:I21"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="12.5703125" style="5" bestFit="1" customWidth="1"/>
@@ -864,7 +855,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="2" spans="1:9" ht="90" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:9" ht="90" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>9</v>
       </c>
@@ -889,7 +880,7 @@
       <c r="H2" s="1"/>
       <c r="I2" s="1"/>
     </row>
-    <row r="3" spans="1:9" ht="135" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:9" ht="135" x14ac:dyDescent="0.25">
       <c r="A3" s="10" t="s">
         <v>16</v>
       </c>
@@ -899,7 +890,7 @@
       <c r="C3" s="10" t="s">
         <v>11</v>
       </c>
-      <c r="D3" s="10" t="s">
+      <c r="D3" s="12" t="s">
         <v>12</v>
       </c>
       <c r="E3" s="10" t="s">
@@ -914,7 +905,7 @@
       <c r="H3" s="10"/>
       <c r="I3" s="10"/>
     </row>
-    <row r="4" spans="1:9" ht="105" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:9" ht="105" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
         <v>20</v>
       </c>
@@ -941,7 +932,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="5" spans="1:9" ht="75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:9" ht="75" x14ac:dyDescent="0.25">
       <c r="A5" s="10" t="s">
         <v>27</v>
       </c>
@@ -968,7 +959,7 @@
       </c>
       <c r="I5" s="10"/>
     </row>
-    <row r="6" spans="1:9" ht="45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:9" ht="45" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
         <v>34</v>
       </c>
@@ -993,7 +984,7 @@
       <c r="H6" s="8"/>
       <c r="I6" s="1"/>
     </row>
-    <row r="7" spans="1:9" ht="90" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:9" ht="120" x14ac:dyDescent="0.25">
       <c r="A7" s="6" t="s">
         <v>40</v>
       </c>
@@ -1001,16 +992,16 @@
         <v>41</v>
       </c>
       <c r="C7" s="6" t="s">
-        <v>11</v>
+        <v>22</v>
       </c>
       <c r="D7" s="6" t="s">
         <v>12</v>
       </c>
       <c r="E7" s="6" t="s">
-        <v>42</v>
+        <v>90</v>
       </c>
       <c r="F7" s="6" t="s">
-        <v>43</v>
+        <v>89</v>
       </c>
       <c r="G7" s="6" t="s">
         <v>15</v>
@@ -1018,12 +1009,12 @@
       <c r="H7" s="6"/>
       <c r="I7" s="6"/>
     </row>
-    <row r="8" spans="1:9" ht="135" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="10" t="s">
-        <v>44</v>
+    <row r="8" spans="1:9" ht="135" x14ac:dyDescent="0.25">
+      <c r="A8" s="9" t="s">
+        <v>42</v>
       </c>
       <c r="B8" s="10" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="C8" s="10" t="s">
         <v>11</v>
@@ -1032,37 +1023,37 @@
         <v>12</v>
       </c>
       <c r="E8" s="10" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="F8" s="10" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="G8" s="10" t="s">
         <v>32</v>
       </c>
       <c r="H8" s="10" t="s">
+        <v>46</v>
+      </c>
+      <c r="I8" s="9"/>
+    </row>
+    <row r="9" spans="1:9" ht="90" x14ac:dyDescent="0.25">
+      <c r="A9" s="6" t="s">
+        <v>47</v>
+      </c>
+      <c r="B9" s="6" t="s">
         <v>48</v>
       </c>
-      <c r="I8" s="9"/>
-    </row>
-    <row r="9" spans="1:9" ht="90" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="6" t="s">
-        <v>49</v>
-      </c>
-      <c r="B9" s="6" t="s">
-        <v>50</v>
-      </c>
       <c r="C9" s="6" t="s">
-        <v>11</v>
+        <v>22</v>
       </c>
       <c r="D9" s="6" t="s">
         <v>23</v>
       </c>
       <c r="E9" s="6" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="F9" s="6" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="G9" s="10" t="s">
         <v>15</v>
@@ -1070,12 +1061,12 @@
       <c r="H9" s="6"/>
       <c r="I9" s="6"/>
     </row>
-    <row r="10" spans="1:9" ht="90" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:9" ht="75" x14ac:dyDescent="0.25">
       <c r="A10" s="10" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="B10" s="10" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="C10" s="10" t="s">
         <v>22</v>
@@ -1084,35 +1075,37 @@
         <v>23</v>
       </c>
       <c r="E10" s="10" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="F10" s="10" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="G10" s="6" t="s">
         <v>15</v>
       </c>
       <c r="H10" s="10"/>
-      <c r="I10" s="10"/>
-    </row>
-    <row r="11" spans="1:9" ht="75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="I10" s="10" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9" ht="75" x14ac:dyDescent="0.25">
       <c r="A11" s="6" t="s">
+        <v>55</v>
+      </c>
+      <c r="B11" s="11" t="s">
+        <v>56</v>
+      </c>
+      <c r="C11" s="6" t="s">
+        <v>36</v>
+      </c>
+      <c r="D11" s="6" t="s">
+        <v>84</v>
+      </c>
+      <c r="E11" s="6" t="s">
         <v>57</v>
       </c>
-      <c r="B11" s="12" t="s">
+      <c r="F11" s="6" t="s">
         <v>58</v>
-      </c>
-      <c r="C11" s="6" t="s">
-        <v>11</v>
-      </c>
-      <c r="D11" s="6" t="s">
-        <v>94</v>
-      </c>
-      <c r="E11" s="6" t="s">
-        <v>59</v>
-      </c>
-      <c r="F11" s="6" t="s">
-        <v>60</v>
       </c>
       <c r="G11" s="10" t="s">
         <v>15</v>
@@ -1120,24 +1113,24 @@
       <c r="H11" s="6"/>
       <c r="I11" s="6"/>
     </row>
-    <row r="12" spans="1:9" ht="120" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:9" ht="120" x14ac:dyDescent="0.25">
       <c r="A12" s="10" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="B12" s="10" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="C12" s="10" t="s">
         <v>36</v>
       </c>
-      <c r="D12" s="11" t="s">
+      <c r="D12" s="9" t="s">
         <v>12</v>
       </c>
       <c r="E12" s="10" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="F12" s="10" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="G12" s="6" t="s">
         <v>15</v>
@@ -1145,12 +1138,12 @@
       <c r="H12" s="9"/>
       <c r="I12" s="10"/>
     </row>
-    <row r="13" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A13" s="3" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>66</v>
+        <v>88</v>
       </c>
       <c r="C13" s="3" t="s">
         <v>22</v>
@@ -1159,10 +1152,10 @@
         <v>12</v>
       </c>
       <c r="E13" s="3" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
       <c r="F13" s="3" t="s">
-        <v>93</v>
+        <v>83</v>
       </c>
       <c r="G13" s="3" t="s">
         <v>15</v>
@@ -1170,149 +1163,126 @@
       <c r="H13" s="3"/>
       <c r="I13" s="3"/>
     </row>
-    <row r="14" spans="1:9" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="4" t="s">
+    <row r="14" spans="1:9" ht="105" x14ac:dyDescent="0.25">
+      <c r="A14" s="10" t="s">
+        <v>65</v>
+      </c>
+      <c r="B14" s="10" t="s">
+        <v>86</v>
+      </c>
+      <c r="C14" s="10" t="s">
+        <v>11</v>
+      </c>
+      <c r="D14" s="10" t="s">
+        <v>12</v>
+      </c>
+      <c r="E14" s="10" t="s">
+        <v>67</v>
+      </c>
+      <c r="F14" s="10" t="s">
+        <v>85</v>
+      </c>
+      <c r="G14" s="10" t="s">
+        <v>15</v>
+      </c>
+      <c r="H14" s="10"/>
+      <c r="I14" s="10" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="15" spans="1:9" ht="120" x14ac:dyDescent="0.25">
+      <c r="A15" s="4" t="s">
+        <v>66</v>
+      </c>
+      <c r="B15" s="4" t="s">
+        <v>69</v>
+      </c>
+      <c r="C15" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="D15" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="E15" s="4" t="s">
+        <v>70</v>
+      </c>
+      <c r="F15" s="4" t="s">
+        <v>71</v>
+      </c>
+      <c r="G15" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="H15" s="4"/>
+      <c r="I15" s="4" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="16" spans="1:9" ht="180" x14ac:dyDescent="0.25">
+      <c r="A16" s="12" t="s">
         <v>68</v>
       </c>
-      <c r="B14" s="4" t="s">
-        <v>69</v>
-      </c>
-      <c r="C14" s="4" t="s">
+      <c r="B16" s="12" t="s">
+        <v>73</v>
+      </c>
+      <c r="C16" s="12" t="s">
+        <v>22</v>
+      </c>
+      <c r="D16" s="12" t="s">
+        <v>74</v>
+      </c>
+      <c r="E16" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="F16" s="12" t="s">
+        <v>76</v>
+      </c>
+      <c r="G16" s="12" t="s">
+        <v>77</v>
+      </c>
+      <c r="H16" s="12"/>
+      <c r="I16" s="12" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="17" spans="1:9" ht="120" x14ac:dyDescent="0.25">
+      <c r="A17" s="4" t="s">
+        <v>72</v>
+      </c>
+      <c r="B17" s="4" t="s">
+        <v>79</v>
+      </c>
+      <c r="C17" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="D14" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="E14" s="4" t="s">
-        <v>70</v>
-      </c>
-      <c r="F14" s="4" t="s">
-        <v>71</v>
-      </c>
-      <c r="G14" s="4" t="s">
-        <v>32</v>
-      </c>
-      <c r="H14" s="4" t="s">
-        <v>72</v>
-      </c>
-      <c r="I14" s="4"/>
-    </row>
-    <row r="15" spans="1:9" ht="120" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="10" t="s">
-        <v>73</v>
-      </c>
-      <c r="B15" s="10" t="s">
-        <v>74</v>
-      </c>
-      <c r="C15" s="10" t="s">
-        <v>11</v>
-      </c>
-      <c r="D15" s="10" t="s">
-        <v>12</v>
-      </c>
-      <c r="E15" s="10" t="s">
-        <v>75</v>
-      </c>
-      <c r="F15" s="10" t="s">
-        <v>76</v>
-      </c>
-      <c r="G15" s="10" t="s">
+      <c r="D17" s="4" t="s">
+        <v>80</v>
+      </c>
+      <c r="E17" s="4" t="s">
+        <v>81</v>
+      </c>
+      <c r="F17" s="4" t="s">
+        <v>82</v>
+      </c>
+      <c r="G17" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="H15" s="10"/>
-      <c r="I15" s="10"/>
-    </row>
-    <row r="16" spans="1:9" ht="120" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="4" t="s">
-        <v>77</v>
-      </c>
-      <c r="B16" s="4" t="s">
-        <v>78</v>
-      </c>
-      <c r="C16" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="D16" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="E16" s="4" t="s">
-        <v>79</v>
-      </c>
-      <c r="F16" s="4" t="s">
-        <v>80</v>
-      </c>
-      <c r="G16" s="4" t="s">
-        <v>15</v>
-      </c>
-      <c r="H16" s="4"/>
-      <c r="I16" s="4"/>
-    </row>
-    <row r="17" spans="1:9" ht="195" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="10" t="s">
-        <v>81</v>
-      </c>
-      <c r="B17" s="10" t="s">
-        <v>82</v>
-      </c>
-      <c r="C17" s="10" t="s">
-        <v>22</v>
-      </c>
-      <c r="D17" s="10" t="s">
-        <v>83</v>
-      </c>
-      <c r="E17" s="10" t="s">
-        <v>84</v>
-      </c>
-      <c r="F17" s="10" t="s">
-        <v>85</v>
-      </c>
-      <c r="G17" s="10" t="s">
-        <v>86</v>
-      </c>
-      <c r="H17" s="10"/>
-      <c r="I17" s="10" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="18" spans="1:9" ht="120" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="4" t="s">
-        <v>88</v>
-      </c>
-      <c r="B18" s="4" t="s">
-        <v>89</v>
-      </c>
-      <c r="C18" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="D18" s="4" t="s">
-        <v>90</v>
-      </c>
-      <c r="E18" s="4" t="s">
-        <v>91</v>
-      </c>
-      <c r="F18" s="4" t="s">
-        <v>92</v>
-      </c>
-      <c r="G18" s="4" t="s">
-        <v>15</v>
-      </c>
-      <c r="H18" s="4"/>
-      <c r="I18" s="4"/>
-    </row>
-    <row r="20" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="E20" s="7"/>
+      <c r="H17" s="4"/>
+      <c r="I17" s="4"/>
+    </row>
+    <row r="18" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="E18" s="7"/>
+    </row>
+    <row r="19" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="H19" s="7"/>
+      <c r="I19" s="7"/>
     </row>
     <row r="21" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="H21" s="7"/>
-      <c r="I21" s="7"/>
-    </row>
-    <row r="23" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="E23" s="7"/>
+      <c r="E21" s="7"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:I1" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
-  <conditionalFormatting sqref="C2:C3 C4:F4 C5:C18 D6:F6">
-    <cfRule type="colorScale" priority="5">
+  <conditionalFormatting sqref="C2:C3 C4:F4 C5:C17 D6:F6">
+    <cfRule type="colorScale" priority="6">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -1328,16 +1298,16 @@
       <formula>NOT(ISERROR(SEARCH("Pass",G1)))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G2:G18">
+  <conditionalFormatting sqref="G2:G17">
     <cfRule type="containsText" dxfId="0" priority="2" operator="containsText" text="Fail">
       <formula>NOT(ISERROR(SEARCH("Fail",G2)))</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C2:C18" xr:uid="{00000000-0002-0000-0000-000000000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C2:C17" xr:uid="{00000000-0002-0000-0000-000000000000}">
       <formula1>"High, Mid, Low"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G2:G18" xr:uid="{00000000-0002-0000-0000-000001000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G2:G17" xr:uid="{00000000-0002-0000-0000-000001000000}">
       <formula1>"Pass, Fail, N/T"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Test Cases Finished + Tool Developed + fix for CMD coments
</commit_message>
<xml_diff>
--- a/1-Manual Test Plans/PARADOX Website Test Plan – Version 1.0.xlsx
+++ b/1-Manual Test Plans/PARADOX Website Test Plan – Version 1.0.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\dario\Documents\GitHub\ParadoxQATest_DarioSC\1-Manual Test Plans\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{498684E7-CF3C-4236-A0A3-8A9981E1ABDA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FCC88FC7-7CD5-404A-8FA5-5984FD8E1263}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="TestPlan-NoLogIn" sheetId="1" r:id="rId1"/>
@@ -87,25 +87,6 @@
     <t>Cookie settings test</t>
   </si>
   <si>
-    <t>1.- Open [https://www.paradoxinteractive.com/our-games/discover]
-2.- Click into the bottom-left [🍪 Cookie settings] button
-     2.1.-Switch on/off the Targeting Cookies
-     2.2.-Switch on/off the Performance Cookies
-     2.3.-Switch on/off the Functional Cookies
-3.- Close the [Cookie settings] sidebar by the following methods
-     3.1.-Click in [Reject All]
-     3.2.-Click in [Confirm My Choices]
-     3.3.-Click in the [X] button upper right</t>
-  </si>
-  <si>
-    <t>2.- A sidebar will open showing the current cookie settings
-     2.1. &amp; 2.2 &amp; 2.3.- The toggles will function normally
-3.- The sidebar will disappear, returning to the Discover site
-     3.1.- The sidebar will disappear with the toggles switched off
-     3.2.- The current toggle selection will be saved and the sidebar will close
-     3.3.- The sidebar will close without saving any changes</t>
-  </si>
-  <si>
     <t>Discover_03</t>
   </si>
   <si>
@@ -258,9 +239,6 @@
 2.- Scroll down until the games list ends and click the image that contains a red title with the text "ON SALE"
 3.- Open [https://www.paradoxinteractive.com/our-games/all-games]
 4.- Scroll down until the game list ends and click the button [SHOP SALE NOW]</t>
-  </si>
-  <si>
-    <t>2. &amp; 4.- The On Sale page will open normally</t>
   </si>
   <si>
     <t>OnSale_01</t>
@@ -388,12 +366,37 @@
 4.- Click into the [SEARCH] bar and write the name of a PARADOX game (repeat this step for five times with PARADOX games)
 5.- Add all the searched games to the cart</t>
   </si>
+  <si>
+    <t>2. &amp; 4.- The On Sale site will open</t>
+  </si>
+  <si>
+    <t>1.- Open [https://www.paradoxinteractive.com/our-games/discover]
+2.- Click into the bottom-left [🍪 Cookie settings] button
+     2.1.- Switch on/off the Targeting Cookies
+     2.2.- Switch on/off the Performance Cookies
+     2.3.- Switch on/off the Functional Cookies
+     2.4.- Switch off the three toggles
+     2.5.- Click in [Allow All]
+3.- Close the [Cookie settings] sidebar by the following methods
+     3.1.- Click in [Reject All]
+     3.2.- Click in [Confirm My Choices]
+     3.3.- Click in the [X] button upper right</t>
+  </si>
+  <si>
+    <t>2.- A sidebar will open showing the current cookie settings
+     2.1. &amp; 2.2 &amp; 2.3. &amp; 2.4.- The toggles will function normally and when it is off the button [Allow All] will appear
+     2.5.- All the toggles will switch on and the sidebar will disappear
+3.- The sidebar will disappear, returning to the Discover site
+     3.1.- The sidebar will disappear with the toggles switched off
+     3.2.- The current toggle selection will be saved and the sidebar will close
+     3.3.- The sidebar will close without saving any changes</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -403,14 +406,6 @@
     </font>
     <font>
       <b/>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <u/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -477,42 +472,27 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -810,474 +790,464 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:I21"/>
+  <dimension ref="A1:I17"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="12.5703125" style="5" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="25.42578125" style="5" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="10.140625" style="5" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="34.140625" style="5" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="64" style="5" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="61.7109375" style="5" customWidth="1"/>
-    <col min="7" max="7" width="9" style="5" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="15.7109375" style="5" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="40.140625" style="5" customWidth="1"/>
-    <col min="10" max="11" width="9.140625" style="5" customWidth="1"/>
-    <col min="12" max="16384" width="9.140625" style="5"/>
+    <col min="1" max="1" width="12.5703125" style="4" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="25.42578125" style="4" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="10.140625" style="4" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="34.140625" style="4" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="64" style="4" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="61.7109375" style="4" customWidth="1"/>
+    <col min="7" max="7" width="9" style="4" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="15.7109375" style="4" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="40.140625" style="4" customWidth="1"/>
+    <col min="10" max="11" width="9.140625" style="4" customWidth="1"/>
+    <col min="12" max="16384" width="9.140625" style="4"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A1" s="2" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="2" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="2" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="2" t="s">
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="2" t="s">
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="2" spans="1:9" ht="90" x14ac:dyDescent="0.25">
-      <c r="A2" s="1" t="s">
+      <c r="A2" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="B2" s="1" t="s">
+      <c r="B2" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="C2" s="1" t="s">
+      <c r="C2" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="D2" s="1" t="s">
+      <c r="D2" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="E2" s="1" t="s">
+      <c r="E2" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="F2" s="1" t="s">
+      <c r="F2" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="G2" s="1" t="s">
+      <c r="G2" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="H2" s="1"/>
-      <c r="I2" s="1"/>
-    </row>
-    <row r="3" spans="1:9" ht="135" x14ac:dyDescent="0.25">
-      <c r="A3" s="10" t="s">
+      <c r="H2" s="5"/>
+      <c r="I2" s="5"/>
+    </row>
+    <row r="3" spans="1:9" ht="165" x14ac:dyDescent="0.25">
+      <c r="A3" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="B3" s="10" t="s">
+      <c r="B3" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="C3" s="10" t="s">
+      <c r="C3" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="D3" s="12" t="s">
+      <c r="D3" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="E3" s="10" t="s">
+      <c r="E3" s="3" t="s">
+        <v>89</v>
+      </c>
+      <c r="F3" s="3" t="s">
+        <v>90</v>
+      </c>
+      <c r="G3" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="H3" s="3"/>
+      <c r="I3" s="3"/>
+    </row>
+    <row r="4" spans="1:9" ht="105" x14ac:dyDescent="0.25">
+      <c r="A4" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="F3" s="10" t="s">
+      <c r="B4" s="5" t="s">
         <v>19</v>
       </c>
-      <c r="G3" s="10" t="s">
+      <c r="C4" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="D4" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="E4" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="F4" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="G4" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="H3" s="10"/>
-      <c r="I3" s="10"/>
-    </row>
-    <row r="4" spans="1:9" ht="105" x14ac:dyDescent="0.25">
-      <c r="A4" s="1" t="s">
+      <c r="H4" s="5"/>
+      <c r="I4" s="5" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" ht="75" x14ac:dyDescent="0.25">
+      <c r="A5" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="B5" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="C5" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="B4" s="1" t="s">
+      <c r="D5" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="E5" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="F5" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="G5" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="H5" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="I5" s="3"/>
+    </row>
+    <row r="6" spans="1:9" ht="45" x14ac:dyDescent="0.25">
+      <c r="A6" s="5" t="s">
+        <v>32</v>
+      </c>
+      <c r="B6" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="C6" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="D6" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="E6" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="F6" s="5" t="s">
+        <v>37</v>
+      </c>
+      <c r="G6" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="H6" s="5"/>
+      <c r="I6" s="5"/>
+    </row>
+    <row r="7" spans="1:9" ht="120" x14ac:dyDescent="0.25">
+      <c r="A7" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="D7" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="E7" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="F7" s="2" t="s">
+        <v>86</v>
+      </c>
+      <c r="G7" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="H7" s="2"/>
+      <c r="I7" s="2"/>
+    </row>
+    <row r="8" spans="1:9" ht="135" x14ac:dyDescent="0.25">
+      <c r="A8" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="B8" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="C8" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="D8" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="E8" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="F8" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="G8" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="H8" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="I8" s="3"/>
+    </row>
+    <row r="9" spans="1:9" ht="90" x14ac:dyDescent="0.25">
+      <c r="A9" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="C9" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="D9" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="C4" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="D4" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="E4" s="1" t="s">
-        <v>24</v>
-      </c>
-      <c r="F4" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="G4" s="1" t="s">
+      <c r="E9" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="F9" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="G9" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="H4" s="1"/>
-      <c r="I4" s="1" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="5" spans="1:9" ht="75" x14ac:dyDescent="0.25">
-      <c r="A5" s="10" t="s">
-        <v>27</v>
-      </c>
-      <c r="B5" s="10" t="s">
-        <v>28</v>
-      </c>
-      <c r="C5" s="10" t="s">
-        <v>22</v>
-      </c>
-      <c r="D5" s="10" t="s">
-        <v>29</v>
-      </c>
-      <c r="E5" s="10" t="s">
-        <v>30</v>
-      </c>
-      <c r="F5" s="10" t="s">
-        <v>31</v>
-      </c>
-      <c r="G5" s="10" t="s">
-        <v>32</v>
-      </c>
-      <c r="H5" s="10" t="s">
-        <v>33</v>
-      </c>
-      <c r="I5" s="10"/>
-    </row>
-    <row r="6" spans="1:9" ht="45" x14ac:dyDescent="0.25">
-      <c r="A6" s="1" t="s">
+      <c r="H9" s="2"/>
+      <c r="I9" s="2"/>
+    </row>
+    <row r="10" spans="1:9" ht="75" x14ac:dyDescent="0.25">
+      <c r="A10" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="B10" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="C10" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="D10" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="E10" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="F10" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="G10" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="H10" s="3"/>
+      <c r="I10" s="3" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9" ht="75" x14ac:dyDescent="0.25">
+      <c r="A11" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="B11" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="C11" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="B6" s="1" t="s">
-        <v>35</v>
-      </c>
-      <c r="C6" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="D6" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="E6" s="1" t="s">
-        <v>38</v>
-      </c>
-      <c r="F6" s="1" t="s">
-        <v>39</v>
-      </c>
-      <c r="G6" s="1" t="s">
+      <c r="D11" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="E11" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="F11" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="G11" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="H6" s="8"/>
-      <c r="I6" s="1"/>
-    </row>
-    <row r="7" spans="1:9" ht="120" x14ac:dyDescent="0.25">
-      <c r="A7" s="6" t="s">
-        <v>40</v>
-      </c>
-      <c r="B7" s="6" t="s">
-        <v>41</v>
-      </c>
-      <c r="C7" s="6" t="s">
-        <v>22</v>
-      </c>
-      <c r="D7" s="6" t="s">
+      <c r="H11" s="2"/>
+      <c r="I11" s="2"/>
+    </row>
+    <row r="12" spans="1:9" ht="120" x14ac:dyDescent="0.25">
+      <c r="A12" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="B12" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="C12" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="D12" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="E7" s="6" t="s">
-        <v>90</v>
-      </c>
-      <c r="F7" s="6" t="s">
-        <v>89</v>
-      </c>
-      <c r="G7" s="6" t="s">
+      <c r="E12" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="F12" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="G12" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="H7" s="6"/>
-      <c r="I7" s="6"/>
-    </row>
-    <row r="8" spans="1:9" ht="135" x14ac:dyDescent="0.25">
-      <c r="A8" s="9" t="s">
-        <v>42</v>
-      </c>
-      <c r="B8" s="10" t="s">
-        <v>43</v>
-      </c>
-      <c r="C8" s="10" t="s">
+      <c r="H12" s="3"/>
+      <c r="I12" s="3"/>
+    </row>
+    <row r="13" spans="1:9" ht="30" x14ac:dyDescent="0.25">
+      <c r="A13" s="6" t="s">
+        <v>60</v>
+      </c>
+      <c r="B13" s="6" t="s">
+        <v>85</v>
+      </c>
+      <c r="C13" s="6" t="s">
+        <v>20</v>
+      </c>
+      <c r="D13" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="E13" s="6" t="s">
+        <v>61</v>
+      </c>
+      <c r="F13" s="6" t="s">
+        <v>80</v>
+      </c>
+      <c r="G13" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="H13" s="6"/>
+      <c r="I13" s="6"/>
+    </row>
+    <row r="14" spans="1:9" ht="105" x14ac:dyDescent="0.25">
+      <c r="A14" s="3" t="s">
+        <v>62</v>
+      </c>
+      <c r="B14" s="3" t="s">
+        <v>83</v>
+      </c>
+      <c r="C14" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="D8" s="10" t="s">
+      <c r="D14" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="E8" s="10" t="s">
-        <v>44</v>
-      </c>
-      <c r="F8" s="10" t="s">
-        <v>45</v>
-      </c>
-      <c r="G8" s="10" t="s">
-        <v>32</v>
-      </c>
-      <c r="H8" s="10" t="s">
-        <v>46</v>
-      </c>
-      <c r="I8" s="9"/>
-    </row>
-    <row r="9" spans="1:9" ht="90" x14ac:dyDescent="0.25">
-      <c r="A9" s="6" t="s">
-        <v>47</v>
-      </c>
-      <c r="B9" s="6" t="s">
-        <v>48</v>
-      </c>
-      <c r="C9" s="6" t="s">
-        <v>22</v>
-      </c>
-      <c r="D9" s="6" t="s">
-        <v>23</v>
-      </c>
-      <c r="E9" s="6" t="s">
-        <v>49</v>
-      </c>
-      <c r="F9" s="6" t="s">
-        <v>50</v>
-      </c>
-      <c r="G9" s="10" t="s">
+      <c r="E14" s="3" t="s">
+        <v>64</v>
+      </c>
+      <c r="F14" s="3" t="s">
+        <v>82</v>
+      </c>
+      <c r="G14" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="H9" s="6"/>
-      <c r="I9" s="6"/>
-    </row>
-    <row r="10" spans="1:9" ht="75" x14ac:dyDescent="0.25">
-      <c r="A10" s="10" t="s">
-        <v>51</v>
-      </c>
-      <c r="B10" s="10" t="s">
-        <v>52</v>
-      </c>
-      <c r="C10" s="10" t="s">
-        <v>22</v>
-      </c>
-      <c r="D10" s="10" t="s">
-        <v>23</v>
-      </c>
-      <c r="E10" s="10" t="s">
-        <v>53</v>
-      </c>
-      <c r="F10" s="10" t="s">
-        <v>54</v>
-      </c>
-      <c r="G10" s="6" t="s">
+      <c r="H14" s="3"/>
+      <c r="I14" s="3" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="15" spans="1:9" ht="120" x14ac:dyDescent="0.25">
+      <c r="A15" s="7" t="s">
+        <v>63</v>
+      </c>
+      <c r="B15" s="7" t="s">
+        <v>66</v>
+      </c>
+      <c r="C15" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="D15" s="7" t="s">
+        <v>12</v>
+      </c>
+      <c r="E15" s="7" t="s">
+        <v>67</v>
+      </c>
+      <c r="F15" s="7" t="s">
+        <v>68</v>
+      </c>
+      <c r="G15" s="7" t="s">
         <v>15</v>
       </c>
-      <c r="H10" s="10"/>
-      <c r="I10" s="10" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="11" spans="1:9" ht="75" x14ac:dyDescent="0.25">
-      <c r="A11" s="6" t="s">
-        <v>55</v>
-      </c>
-      <c r="B11" s="11" t="s">
-        <v>56</v>
-      </c>
-      <c r="C11" s="6" t="s">
-        <v>36</v>
-      </c>
-      <c r="D11" s="6" t="s">
+      <c r="H15" s="7"/>
+      <c r="I15" s="7" t="s">
         <v>84</v>
       </c>
-      <c r="E11" s="6" t="s">
-        <v>57</v>
-      </c>
-      <c r="F11" s="6" t="s">
-        <v>58</v>
-      </c>
-      <c r="G11" s="10" t="s">
+    </row>
+    <row r="16" spans="1:9" ht="180" x14ac:dyDescent="0.25">
+      <c r="A16" s="3" t="s">
+        <v>65</v>
+      </c>
+      <c r="B16" s="3" t="s">
+        <v>70</v>
+      </c>
+      <c r="C16" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="D16" s="3" t="s">
+        <v>71</v>
+      </c>
+      <c r="E16" s="3" t="s">
+        <v>72</v>
+      </c>
+      <c r="F16" s="3" t="s">
+        <v>73</v>
+      </c>
+      <c r="G16" s="3" t="s">
+        <v>74</v>
+      </c>
+      <c r="H16" s="3"/>
+      <c r="I16" s="3" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="17" spans="1:9" ht="120" x14ac:dyDescent="0.25">
+      <c r="A17" s="7" t="s">
+        <v>69</v>
+      </c>
+      <c r="B17" s="7" t="s">
+        <v>76</v>
+      </c>
+      <c r="C17" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="D17" s="7" t="s">
+        <v>77</v>
+      </c>
+      <c r="E17" s="7" t="s">
+        <v>78</v>
+      </c>
+      <c r="F17" s="7" t="s">
+        <v>79</v>
+      </c>
+      <c r="G17" s="7" t="s">
         <v>15</v>
       </c>
-      <c r="H11" s="6"/>
-      <c r="I11" s="6"/>
-    </row>
-    <row r="12" spans="1:9" ht="120" x14ac:dyDescent="0.25">
-      <c r="A12" s="10" t="s">
-        <v>59</v>
-      </c>
-      <c r="B12" s="10" t="s">
-        <v>60</v>
-      </c>
-      <c r="C12" s="10" t="s">
-        <v>36</v>
-      </c>
-      <c r="D12" s="9" t="s">
-        <v>12</v>
-      </c>
-      <c r="E12" s="10" t="s">
-        <v>61</v>
-      </c>
-      <c r="F12" s="10" t="s">
-        <v>62</v>
-      </c>
-      <c r="G12" s="6" t="s">
-        <v>15</v>
-      </c>
-      <c r="H12" s="9"/>
-      <c r="I12" s="10"/>
-    </row>
-    <row r="13" spans="1:9" ht="30" x14ac:dyDescent="0.25">
-      <c r="A13" s="3" t="s">
-        <v>63</v>
-      </c>
-      <c r="B13" s="3" t="s">
-        <v>88</v>
-      </c>
-      <c r="C13" s="3" t="s">
-        <v>22</v>
-      </c>
-      <c r="D13" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="E13" s="3" t="s">
-        <v>64</v>
-      </c>
-      <c r="F13" s="3" t="s">
-        <v>83</v>
-      </c>
-      <c r="G13" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="H13" s="3"/>
-      <c r="I13" s="3"/>
-    </row>
-    <row r="14" spans="1:9" ht="105" x14ac:dyDescent="0.25">
-      <c r="A14" s="10" t="s">
-        <v>65</v>
-      </c>
-      <c r="B14" s="10" t="s">
-        <v>86</v>
-      </c>
-      <c r="C14" s="10" t="s">
-        <v>11</v>
-      </c>
-      <c r="D14" s="10" t="s">
-        <v>12</v>
-      </c>
-      <c r="E14" s="10" t="s">
-        <v>67</v>
-      </c>
-      <c r="F14" s="10" t="s">
-        <v>85</v>
-      </c>
-      <c r="G14" s="10" t="s">
-        <v>15</v>
-      </c>
-      <c r="H14" s="10"/>
-      <c r="I14" s="10" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="15" spans="1:9" ht="120" x14ac:dyDescent="0.25">
-      <c r="A15" s="4" t="s">
-        <v>66</v>
-      </c>
-      <c r="B15" s="4" t="s">
-        <v>69</v>
-      </c>
-      <c r="C15" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="D15" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="E15" s="4" t="s">
-        <v>70</v>
-      </c>
-      <c r="F15" s="4" t="s">
-        <v>71</v>
-      </c>
-      <c r="G15" s="4" t="s">
-        <v>15</v>
-      </c>
-      <c r="H15" s="4"/>
-      <c r="I15" s="4" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="16" spans="1:9" ht="180" x14ac:dyDescent="0.25">
-      <c r="A16" s="12" t="s">
-        <v>68</v>
-      </c>
-      <c r="B16" s="12" t="s">
-        <v>73</v>
-      </c>
-      <c r="C16" s="12" t="s">
-        <v>22</v>
-      </c>
-      <c r="D16" s="12" t="s">
-        <v>74</v>
-      </c>
-      <c r="E16" s="12" t="s">
-        <v>75</v>
-      </c>
-      <c r="F16" s="12" t="s">
-        <v>76</v>
-      </c>
-      <c r="G16" s="12" t="s">
-        <v>77</v>
-      </c>
-      <c r="H16" s="12"/>
-      <c r="I16" s="12" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="17" spans="1:9" ht="120" x14ac:dyDescent="0.25">
-      <c r="A17" s="4" t="s">
-        <v>72</v>
-      </c>
-      <c r="B17" s="4" t="s">
-        <v>79</v>
-      </c>
-      <c r="C17" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="D17" s="4" t="s">
-        <v>80</v>
-      </c>
-      <c r="E17" s="4" t="s">
-        <v>81</v>
-      </c>
-      <c r="F17" s="4" t="s">
-        <v>82</v>
-      </c>
-      <c r="G17" s="4" t="s">
-        <v>15</v>
-      </c>
-      <c r="H17" s="4"/>
-      <c r="I17" s="4"/>
-    </row>
-    <row r="18" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="E18" s="7"/>
-    </row>
-    <row r="19" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="H19" s="7"/>
-      <c r="I19" s="7"/>
-    </row>
-    <row r="21" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="E21" s="7"/>
+      <c r="H17" s="7"/>
+      <c r="I17" s="7"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:I1" xr:uid="{00000000-0009-0000-0000-000000000000}"/>

</xml_diff>